<commit_message>
Made plots in sizing funcitons more usefull and actually work Adresses #20
</commit_message>
<xml_diff>
--- a/MotorSizingFunctions/Parramers.xlsx
+++ b/MotorSizingFunctions/Parramers.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hydra\MQP\MotorSizingFunctions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94E4A783-D1FF-4C63-B009-4FCC907AC1D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91E6E1D7-F88B-4918-AA82-7A5C928F0C56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{E941F4AF-828A-4FA1-8230-FCBA3C5D3139}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>k_m</t>
   </si>
@@ -75,13 +75,58 @@
   </si>
   <si>
     <t>AdditionalPowerDrawsW</t>
+  </si>
+  <si>
+    <t>3S 2200mAh</t>
+  </si>
+  <si>
+    <t>4S 1500mAh</t>
+  </si>
+  <si>
+    <t>4S 1300mAh</t>
+  </si>
+  <si>
+    <t>6S 1100mAh</t>
+  </si>
+  <si>
+    <t>5043 Tri-Blade</t>
+  </si>
+  <si>
+    <t>5045 Dual-Blade</t>
+  </si>
+  <si>
+    <t>6040 Dual-Blade</t>
+  </si>
+  <si>
+    <t>7040 Tri-Blade</t>
+  </si>
+  <si>
+    <t>2205 2300KV</t>
+  </si>
+  <si>
+    <t>2207 2400KV</t>
+  </si>
+  <si>
+    <t>2306 1750KV</t>
+  </si>
+  <si>
+    <t>1806 2280KV</t>
+  </si>
+  <si>
+    <t>Battery Mass</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Total Propeller Mass (all4)</t>
+  </si>
+  <si>
+    <t>Total Motor Weight (all4)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -117,6 +162,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -124,12 +175,6 @@
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="1"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -161,8 +206,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -179,21 +230,95 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -535,115 +660,289 @@
     <col min="2" max="2" width="12.81640625" customWidth="1"/>
     <col min="3" max="3" width="19.81640625" customWidth="1"/>
     <col min="4" max="4" width="16.6328125" customWidth="1"/>
-    <col min="5" max="5" width="4.26953125" customWidth="1"/>
+    <col min="5" max="5" width="12.36328125" customWidth="1"/>
     <col min="6" max="6" width="14.36328125" customWidth="1"/>
-    <col min="9" max="9" width="4.90625" customWidth="1"/>
+    <col min="9" max="9" width="23.1796875" customWidth="1"/>
     <col min="10" max="10" width="12.81640625" customWidth="1"/>
-    <col min="14" max="14" width="5.08984375" customWidth="1"/>
+    <col min="14" max="14" width="19.81640625" customWidth="1"/>
     <col min="15" max="15" width="25.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="1"/>
-      <c r="F1" s="6" t="s">
+      <c r="E1" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="F1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="3" t="s">
+      <c r="G1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="1"/>
-      <c r="J1" s="7" t="s">
+      <c r="I1" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="J1" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="N1" s="1"/>
-      <c r="O1" s="9" t="s">
+      <c r="N1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="O1" s="8" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="E2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="N2" s="1"/>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="E3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="N3" s="1"/>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="E4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="N4" s="1"/>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="E5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="N5" s="1"/>
+    <row r="2" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="10">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C2" s="10">
+        <v>11.1</v>
+      </c>
+      <c r="D2" s="12">
+        <v>1</v>
+      </c>
+      <c r="E2" s="14">
+        <v>0</v>
+      </c>
+      <c r="F2" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="10">
+        <v>1.4999999999999999E-7</v>
+      </c>
+      <c r="H2" s="12">
+        <v>1.1E-5</v>
+      </c>
+      <c r="I2" s="14">
+        <v>0</v>
+      </c>
+      <c r="J2" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" s="10">
+        <v>2300</v>
+      </c>
+      <c r="L2" s="10">
+        <v>1.2</v>
+      </c>
+      <c r="M2" s="12">
+        <v>6.5000000000000002E-2</v>
+      </c>
+      <c r="N2" s="17">
+        <v>0</v>
+      </c>
+      <c r="O2" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="C3" s="10">
+        <v>14.8</v>
+      </c>
+      <c r="D3" s="12">
+        <v>2</v>
+      </c>
+      <c r="E3" s="14">
+        <v>0</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="10">
+        <v>1.1999999999999999E-7</v>
+      </c>
+      <c r="H3" s="12">
+        <v>9.5000000000000005E-6</v>
+      </c>
+      <c r="I3" s="14">
+        <v>0</v>
+      </c>
+      <c r="J3" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="K3" s="10">
+        <v>2400</v>
+      </c>
+      <c r="L3" s="10">
+        <v>1.6</v>
+      </c>
+      <c r="M3" s="12">
+        <v>4.4999999999999998E-2</v>
+      </c>
+      <c r="N3" s="17">
+        <v>0</v>
+      </c>
+      <c r="O3" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="10">
+        <v>1.3</v>
+      </c>
+      <c r="C4" s="10">
+        <v>14.8</v>
+      </c>
+      <c r="D4" s="12">
+        <v>3</v>
+      </c>
+      <c r="E4" s="14">
+        <v>0</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="10">
+        <v>2.2000000000000001E-7</v>
+      </c>
+      <c r="H4" s="12">
+        <v>1.5999999999999999E-5</v>
+      </c>
+      <c r="I4" s="14">
+        <v>0</v>
+      </c>
+      <c r="J4" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" s="10">
+        <v>1750</v>
+      </c>
+      <c r="L4" s="10">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="M4" s="12">
+        <v>5.5E-2</v>
+      </c>
+      <c r="N4" s="17">
+        <v>0</v>
+      </c>
+      <c r="O4" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="10">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C5" s="10">
+        <v>22.2</v>
+      </c>
+      <c r="D5" s="12">
+        <v>4</v>
+      </c>
+      <c r="E5" s="14">
+        <v>0</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="G5" s="10">
+        <v>3.4999999999999998E-7</v>
+      </c>
+      <c r="H5" s="12">
+        <v>2.4000000000000001E-5</v>
+      </c>
+      <c r="I5" s="14">
+        <v>0</v>
+      </c>
+      <c r="J5" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="K5" s="10">
+        <v>2280</v>
+      </c>
+      <c r="L5" s="10">
+        <v>0.8</v>
+      </c>
+      <c r="M5" s="12">
+        <v>0.11</v>
+      </c>
+      <c r="N5" s="17">
+        <v>0</v>
+      </c>
+      <c r="O5" s="11">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="E6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="N6" s="1"/>
+      <c r="E6" s="14"/>
+      <c r="I6" s="14"/>
+      <c r="N6" s="17"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="E7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="N7" s="1"/>
+      <c r="E7" s="14"/>
+      <c r="I7" s="14"/>
+      <c r="N7" s="17"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="E8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="N8" s="1"/>
+      <c r="E8" s="14"/>
+      <c r="I8" s="14"/>
+      <c r="N8" s="17"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="E9" s="1"/>
-      <c r="I9" s="1"/>
-      <c r="N9" s="1"/>
+      <c r="E9" s="14"/>
+      <c r="I9" s="14"/>
+      <c r="N9" s="17"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="E10" s="1"/>
-      <c r="I10" s="1"/>
-      <c r="N10" s="1"/>
+      <c r="E10" s="14"/>
+      <c r="I10" s="14"/>
+      <c r="N10" s="17"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A11" s="8"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="1"/>
-      <c r="J11" s="8"/>
-      <c r="K11" s="8"/>
-      <c r="L11" s="8"/>
-      <c r="M11" s="8"/>
-      <c r="N11" s="1"/>
+      <c r="A11" s="7"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="14"/>
+      <c r="J11" s="7"/>
+      <c r="K11" s="7"/>
+      <c r="L11" s="7"/>
+      <c r="M11" s="7"/>
+      <c r="N11" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>